<commit_message>
Recheck Best 14 vs Best 10; show both totals on every league table
Mark Ready verified at 25 rounds: Best 14 = 273, Best 10 = 201.
Headers now say Best 14 pts / Best 10 pts / Rounds to avoid ambiguity.

Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -27,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="£#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,13 +51,19 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001A3A2A"/>
-      <sz val="13"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A3A2A"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="4">
@@ -104,15 +110,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -479,14 +486,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,20 +511,20 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>RS Cup champion: Mark Ready · Champ/Chumps still to play</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Headline winners</t>
-        </is>
-      </c>
-    </row>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RS Cup: Mark Ready beat Simon Carter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CHECK Mark Ready: 25 rounds · Best 14 pts = 273 · Best 10 pts = 201</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -531,20 +538,24 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr"/>
+          <t>Best 14 pts</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Rounds / note</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Best 14</t>
+          <t>Best 14 champion</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -552,43 +563,39 @@
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="5" t="n">
         <v>295</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>24 games</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Best 10 217</t>
-        </is>
+      <c r="D7" s="5" t="n">
+        <v>217</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>RS Cup</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>RS Cup champion</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Final: Simon Carter vs Mark Ready</t>
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Simon Carter vs Mark Ready</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Money</t>
+          <t>Money leader</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -596,32 +603,32 @@
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>1 wins</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Most snakes</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Paul Chapman</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="7" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -634,229 +641,227 @@
           <t>Tim Lewis</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="5" t="inlineStr"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Season stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Season stats</t>
-        </is>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Players</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>66</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Weeks</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n">
+          <t>Avg field</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Players</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>66</v>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Champions</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Avg field</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>28</v>
+          <t>Paid out</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>1176</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Champions</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>13</v>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>To bank</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>3148</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Paid out</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>1176</v>
+          <t>Snakes</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>200</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>To bank</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>3148</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Snakes</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>200</v>
-      </c>
-    </row>
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Camels</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Camels</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="n">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="24"/>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Division winners</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Best 14 pts</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Division winners (Best 10)</t>
-        </is>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Steve Such</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>217</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>295</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Division</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Winner</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Best 14</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Jez Williams</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>213</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>287</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Premiership</t>
+          <t>League One</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Steve Such</t>
+          <t>Mark Jackson</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Jez Williams</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>213</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>287</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Mark Jackson</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>204</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>279</v>
-      </c>
-      <c r="E29" s="5" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C28" s="6" t="n">
         <v>201</v>
       </c>
-      <c r="D30" s="7" t="n">
+      <c r="D28" s="6" t="n">
         <v>255</v>
       </c>
-      <c r="E30" s="7" t="n">
+      <c r="E28" s="6" t="n">
         <v>14</v>
       </c>
     </row>
@@ -874,25 +879,25 @@
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Best 14 — top 15 (club series)</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Best 14 — top 15</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Best 14 = sum of best 14 weekly scores. Best 10 = sum of best 10 (used for leagues). They match only if the player has ≤10 rounds.</t>
+          <t>Best 14 pts = sum of best 14 weekly scores. Best 10 pts = sum of best 10 (league ranking). Rounds = counting weeks played.</t>
         </is>
       </c>
     </row>
@@ -910,17 +915,17 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Best 14</t>
+          <t>Best 14 pts</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Best 10</t>
+          <t>Best 10 pts</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Games</t>
+          <t>Rounds</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -954,24 +959,24 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Jez Williams</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>287</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
@@ -1002,24 +1007,24 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>278</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
@@ -1050,24 +1055,24 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>275</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
@@ -1098,24 +1103,24 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>273</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="6" t="n">
         <v>201</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
@@ -1146,24 +1151,24 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>271</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="6" t="n">
         <v>202</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
@@ -1194,24 +1199,24 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>263</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
@@ -1242,24 +1247,24 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Ian Ind</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="6" t="n">
         <v>262</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="6" t="n">
         <v>193</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="E18" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
@@ -1300,282 +1305,340 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Premiership — ranked by Best 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Premiership — ranked by Best 10 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Best 14 pts shown for reference; league position uses Best 10 pts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Best 14 pts</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C5" s="5" t="n">
         <v>217</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D5" s="5" t="n">
+        <v>295</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>207</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D6" s="6" t="n">
+        <v>277</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C7" s="5" t="n">
         <v>207</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D7" s="5" t="n">
+        <v>273</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>19</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D8" s="6" t="n">
+        <v>275</v>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="5" t="n">
         <v>203</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D9" s="5" t="n">
+        <v>278</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>26</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>199</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D10" s="6" t="n">
+        <v>270</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Tony Mynard</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C11" s="5" t="n">
         <v>196</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D11" s="5" t="n">
+        <v>261</v>
+      </c>
+      <c r="E11" s="5" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Ian Ind</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>193</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D12" s="6" t="n">
+        <v>262</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Dave Harrison</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C13" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D13" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="E13" s="5" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Tim Lewis</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D14" s="6" t="n">
+        <v>251</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Richard Bird</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C15" s="5" t="n">
         <v>184</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D15" s="5" t="n">
+        <v>235</v>
+      </c>
+      <c r="E15" s="5" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Jon Boden</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D16" s="6" t="n">
+        <v>209</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Andy Ray</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C17" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D17" s="5" t="n">
+        <v>199</v>
+      </c>
+      <c r="E17" s="5" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C18" s="6" t="n">
         <v>176</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D18" s="6" t="n">
+        <v>218</v>
+      </c>
+      <c r="E18" s="6" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Tom Green</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C19" s="5" t="n">
         <v>151</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D19" s="5" t="n">
+        <v>173</v>
+      </c>
+      <c r="E19" s="5" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1590,282 +1653,340 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Championship — ranked by Best 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Championship — ranked by Best 10 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Best 14 pts shown for reference; league position uses Best 10 pts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Best 14 pts</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Jez Williams</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C5" s="5" t="n">
         <v>213</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D5" s="5" t="n">
+        <v>287</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>202</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D6" s="6" t="n">
+        <v>271</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>19</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C7" s="5" t="n">
         <v>201</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D7" s="5" t="n">
+        <v>273</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D8" s="6" t="n">
+        <v>272</v>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Martin Stevenson</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="5" t="n">
         <v>194</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D9" s="5" t="n">
+        <v>260</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Kevin Horton</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>191</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D10" s="6" t="n">
+        <v>257</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Mick Sandoz</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C11" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D11" s="5" t="n">
+        <v>249</v>
+      </c>
+      <c r="E11" s="5" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Steve Robinson</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>188</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D12" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C13" s="5" t="n">
         <v>187</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D13" s="5" t="n">
+        <v>220</v>
+      </c>
+      <c r="E13" s="5" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Gary Adcock</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>187</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D14" s="6" t="n">
+        <v>252</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Paul Smith</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C15" s="5" t="n">
         <v>173</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D15" s="5" t="n">
+        <v>197</v>
+      </c>
+      <c r="E15" s="5" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Jon Murchington</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>152</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D16" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Paul Blades</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C17" s="5" t="n">
         <v>133</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D17" s="5" t="n">
+        <v>133</v>
+      </c>
+      <c r="E17" s="5" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Marc Allsopp</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C18" s="6" t="n">
         <v>104</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D18" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="E18" s="6" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Lee Eastoe</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="5" t="n">
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1880,282 +2001,340 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>League One — ranked by Best 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>League One — ranked by Best 10 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Best 14 pts shown for reference; league position uses Best 10 pts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Best 14 pts</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Mark Jackson</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C5" s="5" t="n">
         <v>204</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D5" s="5" t="n">
+        <v>279</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D6" s="6" t="n">
+        <v>263</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C7" s="5" t="n">
         <v>195</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D7" s="5" t="n">
+        <v>261</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>194</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D8" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Ade Cooper</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="5" t="n">
         <v>187</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D9" s="5" t="n">
+        <v>245</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Stuart Murdock</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D10" s="6" t="n">
+        <v>238</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Paul Chapman</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C11" s="5" t="n">
         <v>167</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D11" s="5" t="n">
+        <v>217</v>
+      </c>
+      <c r="E11" s="5" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Les Lawrence</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>162</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D12" s="6" t="n">
+        <v>188</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Stuart Pickersgill</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C13" s="5" t="n">
         <v>158</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D13" s="5" t="n">
+        <v>158</v>
+      </c>
+      <c r="E13" s="5" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Steve Rochester</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>124</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D14" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Richard Craven Jones</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C15" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D15" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="E15" s="5" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Mark Jeffries</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D16" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Ross Jeffries</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Stephen Wallace</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="C18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Stu Clark</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="5" t="n">
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2170,378 +2349,454 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>League Two — ranked by Best 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>League Two — ranked by Best 10 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Best 14 pts shown for reference; league position uses Best 10 pts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Best 14 pts</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C5" s="5" t="n">
         <v>201</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D5" s="5" t="n">
+        <v>255</v>
+      </c>
+      <c r="E5" s="5" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Andrew Mosson</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>199</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D6" s="6" t="n">
+        <v>263</v>
+      </c>
+      <c r="E6" s="6" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Ross Kelly</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C7" s="5" t="n">
         <v>194</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D7" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="E7" s="5" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Dan Conway</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>181</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D8" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
+    <row r="9">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>James Simmons</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="5" t="n">
         <v>170</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D9" s="5" t="n">
+        <v>194</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Mark Mosley</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D10" s="6" t="n">
+        <v>166</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Ashley Wells</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C11" s="5" t="n">
         <v>146</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D11" s="5" t="n">
+        <v>146</v>
+      </c>
+      <c r="E11" s="5" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Andy Spencer</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D12" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="E12" s="6" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Richard Cook</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C13" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D13" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="E13" s="5" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Brian Elliot</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D14" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="E14" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
+    <row r="15">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Mick Hennessy</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C15" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D15" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E15" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Craig Jones</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="C16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Craig Milligan</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>James Willis</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="C18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Jon Price</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Matt Spencer</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="C20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Neale Aston</t>
         </is>
       </c>
-      <c r="C20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Paul Garratt</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="C22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Scott Worrall</t>
         </is>
       </c>
-      <c r="C22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="C23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Steve Tarmey</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="C24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Warren Crook</t>
         </is>
       </c>
-      <c r="C24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="5" t="n">
+      <c r="C25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2556,314 +2811,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>2027 promotion &amp; relegation preview</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Top 3 promote / bottom 3 relegate by Best 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Promoted</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Jez Williams</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Richard Shaw</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jackson</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Adam Simcox</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>James Harrison</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Carl Rowe</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>League Two</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Andrew Mosson</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>League Two</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Ross Kelly</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>League Two</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Relegated</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Mark Jackson</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Best 10 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Andy Ray</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Adam Simcox</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="D17" s="5" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Mark Howell</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>James Harrison</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Carl Rowe</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>League Two</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Andrew Mosson</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>League Two</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Ross Kelly</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>League Two</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Jez Williams</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Richard Shaw</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Relegated</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>From</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>To</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
+      <c r="D18" s="6" t="n">
+        <v>176</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Lee Eastoe</t>
+          <t>Tom Green</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="D19" s="5" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Paul Blades</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Marc Allsopp</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>104</v>
+      <c r="D20" s="6" t="n">
+        <v>133</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Paul Blades</t>
+          <t>Marc Allsopp</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -2877,127 +3164,87 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>133</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Ross Jeffries</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Lee Eastoe</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>League Two</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>Ross Jeffries</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>League Two</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
           <t>Stephen Wallace</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="D23" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Stu Clark</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>League Two</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Tom Green</t>
+          <t>Stu Clark</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Premiership</t>
+          <t>League One</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Championship</t>
+          <t>League Two</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Andy Ray</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Mark Howell</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>176</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3011,19 +3258,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Money leaders (outright weeks)</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Money leaders</t>
         </is>
       </c>
     </row>
@@ -3062,23 +3309,23 @@
       <c r="C4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="7" t="n">
         <v>150</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="9" t="n">
         <v>147</v>
       </c>
     </row>
@@ -3094,23 +3341,23 @@
       <c r="C6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <v>136.5</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>133.5</v>
       </c>
     </row>
@@ -3126,23 +3373,23 @@
       <c r="C8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n">
         <v>88.5</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <v>84</v>
       </c>
     </row>
@@ -3158,23 +3405,23 @@
       <c r="C10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="7" t="n">
         <v>63</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>57</v>
       </c>
     </row>
@@ -3190,205 +3437,203 @@
       <c r="C12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="7" t="n">
         <v>51</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="9" t="n">
         <v>51</v>
       </c>
     </row>
     <row r="14"/>
-    <row r="15"/>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Snakes</t>
+        </is>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Snakes (top 5)</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Count</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Paul Chapman</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Peter Jeffries</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Richard Shaw</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Gary Adcock</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Camels</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
+    <row r="25">
+      <c r="A25" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Paul Chapman</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Tim Lewis</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Ian Ind</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
         <v>11</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Peter Jeffries</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Richard Shaw</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Gary Adcock</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Camels (top 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Tim Lewis</t>
+          <t>Gary Adcock</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Ian Ind</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>11</v>
+      <c r="A28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Gary Adcock</t>
+          <t>Peter Jeffries</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>John Goodman</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Peter Jeffries</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3403,7 +3648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3411,7 +3656,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Champions field</t>
         </is>
@@ -3433,7 +3678,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
@@ -3447,7 +3692,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
@@ -3461,7 +3706,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
@@ -3475,7 +3720,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
@@ -3489,7 +3734,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
@@ -3503,7 +3748,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
@@ -3517,53 +3762,52 @@
       </c>
     </row>
     <row r="17"/>
-    <row r="18"/>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>RS Cup Final</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>RS Cup Final</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Mark Ready beat Simon Carter</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Semi-final</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Winner</t>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Mark Ready vs Steve Such</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Mark Ready vs Steve Such</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Simon Carter vs Ade Cooper</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>

</xml_diff>

<commit_message>
Add away day credits at £1.50 per weekly game played
Credits from Main Summer 2026 finalized weekly appearances; total and
per-player breakdown added to the final-day HTML, PDF and Excel pack.

Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -15,7 +15,8 @@
     <sheet name="League Two" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Promotion &amp; relegation" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Money &amp; wildlife" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Champions &amp; RS Cup" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Away day credits" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Champions &amp; RS Cup" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="£#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +64,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -114,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +131,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,11 +498,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -601,254 +608,457 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Most snakes</t>
+          <t>Away day credits</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Paul Chapman</t>
+          <t>£1176.00 total</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>£1.50 × 784 games</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>Most snakes</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Paul Chapman</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>Most camels</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Tim Lewis</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Season</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Weeks</t>
         </is>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B16" s="8" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Players</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B17" s="9" t="n">
         <v>66</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Average field</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n">
+      <c r="B18" s="8" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Champions</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B19" s="9" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Paid out</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B20" s="8" t="n">
         <v>1176</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>To bank</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B21" s="9" t="n">
         <v>3148</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Snakes</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B22" s="8" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Camels</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B23" s="9" t="n">
         <v>204</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Away day credits</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Division winners</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Winner</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Rounds</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Steve Such</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>217</v>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>295</v>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Jez Williams</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>213</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>287</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>League One</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Mark Jackson</t>
+          <t>Steve Such</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Jez Williams</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>287</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jackson</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>204</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>279</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C31" s="7" t="n">
         <v>201</v>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="D31" s="7" t="n">
         <v>255</v>
       </c>
-      <c r="E29" s="7" t="n">
+      <c r="E31" s="7" t="n">
         <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Champions League field</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Adam Simcox</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Adam Teale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Carl Rowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Chris Boards</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>James Harrison</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>James Tough</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Mark Howell</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Nick Stableford</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Peter Jeffries</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Steve Such</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Tim Allsopp</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>RS Cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Mark Ready beat Simon Carter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Semi-final</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Mark Ready vs Steve Such</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Simon Carter vs Ade Cooper</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Simon Carter</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3599,169 +3809,903 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Champions League field</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Away day credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>£1.50 per weekly game played</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>52 players · 784 games · £1176.00 total</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Tim Allsopp</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Gary Adcock</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Ian Ind</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Chris Boards</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Steve Such</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Tim Lewis</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Peter Jeffries</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Tony Mynard</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Andrew Mosson</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jackson</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Martin Stevenson</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Nick Stableford</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>James Harrison</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Simon Carter</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>James Tough</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Jez Williams</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Richard Shaw</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="C25" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Ade Cooper</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Dave Harrison</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Kevin Horton</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Mick Sandoz</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Paul Chapman</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Richard Bird</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Steve Robinson</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Stuart Murdock</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Carl Rowe</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Mark Howell</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Carl Rowe</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Chris Boards</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>James Harrison</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>James Tough</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>John Goodman</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Mark Howell</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Nick Stableford</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Peter Jeffries</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Steve Such</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Tim Allsopp</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>RS Cup</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Mark Ready beat Simon Carter</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Semi-final</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Winner</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Mark Ready vs Steve Such</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Simon Carter vs Ade Cooper</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Simon Carter</t>
-        </is>
+      <c r="C36" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Dan Conway</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Jon Boden</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Les Lawrence</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Ross Kelly</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Tom Green</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Andy Ray</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>James Simmons</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Paul Smith</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Jon Murchington</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Mark Mosley</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Stuart Pickersgill</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Ashley Wells</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Paul Blades</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Steve Rochester</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Marc Allsopp</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Andy Spencer</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Richard Craven Jones</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Richard Cook</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Brian Elliot</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jeffries</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Mick Hennessy</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="58"/>
+    <row r="59">
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="n">
+        <v>784</v>
+      </c>
+      <c r="D59" s="11" t="n">
+        <v>1176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add money summary: weekly winners, away credits, bank
Separate member payouts (winner pot + £1.50/game credits) from club bank
and show season totals in the final-day pack.

Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -8,15 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="Headlines" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Best 14" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Premiership" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Championship" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="League One" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="League Two" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Promotion &amp; relegation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Money &amp; wildlife" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Away day credits" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Champions &amp; RS Cup" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Money summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Best 14" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Premiership" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Championship" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="League One" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="League Two" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Promotion &amp; relegation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Weekly money leaders" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Away day credits" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Champions &amp; RS Cup" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -75,7 +76,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +91,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F8F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF3EF"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,6 +136,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -498,12 +506,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -608,280 +616,136 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Away day credits</t>
+          <t>Paid to members</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>£1176.00 total</t>
+          <t>£2352.00</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>£1.50 × 784 games</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Most snakes</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Paul Chapman</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-    </row>
+          <t>Winners £1176.00 + credits £1176.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Most camels</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Tim Lewis</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Division winners</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Best 10</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Best 14</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Rounds</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Season</t>
-        </is>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Steve Such</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>217</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>295</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Jez Williams</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>213</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>287</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Weeks</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n">
-        <v>28</v>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jackson</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>204</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>279</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Players</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="n">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Average field</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Champions</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Paid out</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>1176</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>To bank</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n">
-        <v>3148</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Snakes</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Camels</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Away day credits</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n">
-        <v>1176</v>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Division winners</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Division</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Winner</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Best 14</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Rounds</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Steve Such</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>217</v>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>295</v>
-      </c>
-      <c r="E28" s="6" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Jez Williams</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>213</v>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>287</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Mark Jackson</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>204</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>279</v>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C17" s="7" t="n">
         <v>201</v>
       </c>
-      <c r="D31" s="7" t="n">
+      <c r="D17" s="7" t="n">
         <v>255</v>
       </c>
-      <c r="E31" s="7" t="n">
+      <c r="E17" s="7" t="n">
         <v>14</v>
       </c>
     </row>
@@ -891,6 +755,909 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="47" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Away day credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>£1.50 per weekly game played · £1176.00 total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Tim Allsopp</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Gary Adcock</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Ian Ind</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Chris Boards</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Steve Such</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Tim Lewis</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Peter Jeffries</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Tony Mynard</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>34.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Andrew Mosson</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jackson</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Martin Stevenson</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Nick Stableford</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>James Harrison</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Simon Carter</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>James Tough</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Jez Williams</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Richard Shaw</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Adam Simcox</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Ade Cooper</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Dave Harrison</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Kevin Horton</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Mick Sandoz</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Paul Chapman</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Richard Bird</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Steve Robinson</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Stuart Murdock</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Carl Rowe</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Mark Howell</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Adam Teale</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Dan Conway</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Jon Boden</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Les Lawrence</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Ross Kelly</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Tom Green</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Andy Ray</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>James Simmons</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Paul Smith</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Jon Murchington</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Mark Mosley</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Stuart Pickersgill</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Ashley Wells</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Paul Blades</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Steve Rochester</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Marc Allsopp</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Andy Spencer</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Richard Craven Jones</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Richard Cook</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Brian Elliot</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Mark Jeffries</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Mick Hennessy</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="n">
+        <v>784</v>
+      </c>
+      <c r="D58" s="13" t="n">
+        <v>1176</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1018,7 +1785,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>Mark Ready beat Simon Carter</t>
         </is>
@@ -1067,6 +1834,132 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Money summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Main Summer 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Weekly winner payouts</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Paid to outright weekly winners</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Away day credits</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>£1.50 × 784 games played</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Total to members</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Winners + away day credits</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>2352</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Club bank</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>£3.50 per game (£2744.00) + snakes/camels £1 (£404.00)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>3148</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Season total</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Members + club bank</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>5500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1488,7 +2381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1829,7 +2722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2170,7 +3063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2511,7 +3404,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2966,7 +3859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3413,7 +4306,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3422,7 +4315,7 @@
   <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -3431,7 +4324,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Money leaders</t>
+          <t>Weekly money leaders</t>
         </is>
       </c>
     </row>
@@ -3796,916 +4689,6 @@
       </c>
       <c r="C29" s="6" t="n">
         <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D59"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Away day credits</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>£1.50 per weekly game played</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>52 players · 784 games · £1176.00 total</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Credit</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Tim Allsopp</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Gary Adcock</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Ian Ind</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Chris Boards</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Steve Such</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Tim Lewis</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Peter Jeffries</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>34.5</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Tony Mynard</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>34.5</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Andrew Mosson</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Mark Jackson</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Martin Stevenson</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Nick Stableford</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>James Harrison</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>31.5</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Simon Carter</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>31.5</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>James Tough</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Jez Williams</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>John Goodman</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="D23" s="9" t="n">
-        <v>28.5</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Richard Shaw</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="D24" s="8" t="n">
-        <v>28.5</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Adam Simcox</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Ade Cooper</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Dave Harrison</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>17</v>
-      </c>
-      <c r="D27" s="9" t="n">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Kevin Horton</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Mick Sandoz</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="D29" s="9" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Paul Chapman</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Richard Bird</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="D31" s="9" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Steve Robinson</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Stuart Murdock</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="D33" s="9" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Carl Rowe</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="D34" s="8" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Mark Howell</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="D35" s="9" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Adam Teale</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D36" s="8" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Dan Conway</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="D37" s="9" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Jon Boden</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Les Lawrence</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="D39" s="9" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Ross Kelly</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D40" s="8" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Tom Green</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="D41" s="9" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>Andy Ray</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D42" s="8" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="7" t="n">
-        <v>38</v>
-      </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>James Simmons</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D43" s="9" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Paul Smith</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D44" s="8" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Jon Murchington</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D45" s="9" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="6" t="inlineStr">
-        <is>
-          <t>Mark Mosley</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D46" s="8" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Stuart Pickersgill</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D47" s="9" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Ashley Wells</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Paul Blades</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D49" s="9" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Steve Rochester</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D50" s="8" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Marc Allsopp</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D51" s="9" t="n">
-        <v>10.5</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Andy Spencer</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D52" s="8" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="n">
-        <v>48</v>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Richard Craven Jones</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="D53" s="9" t="n">
-        <v>4.5</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Richard Cook</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" s="8" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Brian Elliot</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" s="9" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="n">
-        <v>51</v>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Mark Jeffries</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="8" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="7" t="n">
-        <v>52</v>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>Mick Hennessy</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="9" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="58"/>
-    <row r="59">
-      <c r="B59" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C59" s="10" t="n">
-        <v>784</v>
-      </c>
-      <c r="D59" s="11" t="n">
-        <v>1176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix money summary: Champions payouts vs away day credits
Weekly winner payouts are outright Champions only (£1,095). Away day
credits remain £1.50 per week played (£1,176). Final week split listed separately.

Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -511,7 +511,7 @@
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -626,7 +626,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Winners £1176.00 + credits £1176.00</t>
+          <t>Champions £1095.00 + away £1176.00</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
   <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="47" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -779,7 +779,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>£1.50 per weekly game played · £1176.00 total</t>
+          <t>£1.50 per week played · £1176.00 total</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Games</t>
+          <t>Weeks</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -1839,7 +1839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1887,11 +1887,11 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Paid to outright weekly winners</t>
+          <t>Champions League — outright weekly winners</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>1176</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="6">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>£1.50 × 784 games played</t>
+          <t>£1.50 per week played · 784 games</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
@@ -1910,47 +1910,58 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Final week split</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Shared among top scores — no Champions place</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Total to members</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Winners + away day credits</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="n">
+      <c r="B8" s="10" t="inlineStr"/>
+      <c r="C8" s="11" t="n">
         <v>2352</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Club bank</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>£3.50 per game (£2744.00) + snakes/camels £1 (£404.00)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="n">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>£3.50 per game (£2744.00) + snakes/camels (£404.00)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
         <v>3148</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Season total</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Members + club bank</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C10" s="11" t="n">
         <v>5500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
List all weekly Champions winners, not only top 10
Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -15,9 +15,10 @@
     <sheet name="League One" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="League Two" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Promotion &amp; relegation" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Weekly money leaders" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Away day credits" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Champions &amp; RS Cup" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Weekly winners" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Snakes &amp; camels" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Away day credits" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Champions &amp; RS Cup" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -760,6 +761,205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Snakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Paul Chapman</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Peter Jeffries</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Mark Ready</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Richard Shaw</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Gary Adcock</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Camels</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Tim Lewis</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Ian Ind</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Gary Adcock</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Peter Jeffries</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1657,7 +1857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1839,7 +2039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1854,114 +2054,107 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Main Summer 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Weekly winner payouts</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Champions League — outright weekly winners</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>1095</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Weekly winner payouts</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Champions League — outright weekly winners</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>1095</v>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Away day credits</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>£1.50 per week played · 784 games</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>1176</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Away day credits</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>£1.50 per week played · 784 games</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>1176</v>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Final week split</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Shared among top scores — no Champions place</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Final week split</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Shared among top scores — no Champions place</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>81</v>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Total to members</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr"/>
+      <c r="C7" s="11" t="n">
+        <v>2352</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Total to members</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="n">
-        <v>2352</v>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Club bank</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>£3.50 per game (£2744.00) + snakes/camels (£404.00)</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>3148</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Club bank</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>£3.50 per game (£2744.00) + snakes/camels (£404.00)</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>3148</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Season total</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Members + club bank</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C9" s="11" t="n">
         <v>5500</v>
       </c>
     </row>
@@ -4323,10 +4516,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -4335,371 +4528,260 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Weekly money leaders</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+          <t>Weekly winners</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>All outright Champions · 13 winners · £1095.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="n">
+    <row r="5">
+      <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D5" s="8" t="n">
         <v>150</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="6">
+      <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D6" s="9" t="n">
         <v>147</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
+    <row r="7">
+      <c r="A7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D7" s="8" t="n">
         <v>136.5</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="8">
+      <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D8" s="9" t="n">
         <v>133.5</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
+    <row r="9">
+      <c r="A9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D9" s="8" t="n">
         <v>88.5</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="n">
+    <row r="10">
+      <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D10" s="9" t="n">
         <v>84</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
+    <row r="11">
+      <c r="A11" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D11" s="8" t="n">
         <v>63</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D12" s="9" t="n">
         <v>57</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
+    <row r="13">
+      <c r="A13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D13" s="8" t="n">
         <v>51</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+    <row r="14">
+      <c r="A14" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D14" s="9" t="n">
         <v>51</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Snakes</t>
-        </is>
+      <c r="A15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Tim Allsopp</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>49.5</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
+      <c r="A16" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>John Goodman</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>46.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>James Tough</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Paul Chapman</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Peter Jeffries</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>10</v>
-      </c>
-    </row>
+      <c r="D17" s="8" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Richard Shaw</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Gary Adcock</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Camels</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Tim Lewis</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Ian Ind</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Gary Adcock</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>John Goodman</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Peter Jeffries</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>9</v>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>1095</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix money summary: stop double-counting away credits in season total
Season collections (£5/game + fines) balance to winners + final week + bank.
Away day credits shown separately, not added on top.

Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -512,7 +512,7 @@
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -617,17 +617,17 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Paid to members</t>
+          <t>Away day credits</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>£2352.00</t>
+          <t>£1176.00</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Champions £1095.00 + away £1176.00</t>
+          <t>£1.50 × 784 weeks</t>
         </is>
       </c>
     </row>
@@ -2039,11 +2039,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -2054,108 +2054,145 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Weekly collections balance separately from away day credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Weekly winner payouts</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Champions League — outright weekly winners</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>1095</v>
-      </c>
-    </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Away day credits</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>£1.50 per week played · 784 games</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="n">
-        <v>1176</v>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Entry fees collected</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>£5.00 × 784 games</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>3920</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Final week split</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Shared among top scores — no Champions place</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>81</v>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Snake &amp; camel fines</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>£1.00 × 404</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>404</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Total to members</t>
+          <t>Total collected</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr"/>
       <c r="C7" s="11" t="n">
-        <v>2352</v>
+        <v>4324</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Weekly winner payouts</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Champions League — outright weekly winners</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Final week split</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Shared among top scores — no Champions place</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Club bank</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>£3.50 per game (£2744.00) + snakes/camels (£404.00)</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>£3.50 per game (£2744.00) + fines (£404.00)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
         <v>3148</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Season total</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Members + club bank</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>5500</v>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Allocated from collections</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Winners + final week + bank</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>4324</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Away day credits</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>£1.50 per week played · 784 games</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild final-day presentation from verified live data
Re-checked standings, money collections/allocations, Mark Ready Best 14/10,
RS Cup, all 13 weekly Champions winners, and away day credits.

Co-authored-by: reddii7 <reddii7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/WAGS_2026_Final_Day_Presentation.xlsx
+++ b/WAGS_2026_Final_Day_Presentation.xlsx
@@ -58,14 +58,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001B5C37"/>
-      <sz val="13"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="001B5C37"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -131,10 +131,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -542,211 +542,204 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Headlines</t>
+          <t>Award</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Award</t>
+          <t>Best 14</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Winner</t>
+          <t>Steve Such</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Detail</t>
+          <t>295 points</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Best 14</t>
+          <t>RS Cup</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Steve Such</t>
+          <t>Mark Ready</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>295 points</t>
+          <t>Beat Simon Carter</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>RS Cup</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Mark Ready</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Beat Simon Carter</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Weekly money</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Carl Rowe</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>£150.00 · 1 wins</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Weekly money</t>
+          <t>Away day credits</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Carl Rowe</t>
+          <t>£1176.00</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>£150.00 · 1 win</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Away day credits</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>£1176.00</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
           <t>£1.50 × 784 weeks</t>
         </is>
       </c>
     </row>
-    <row r="11"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Division winners</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Division winners</t>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Best 10</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Best 14</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Rounds</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Division</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Winner</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Best 10</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Best 14</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Rounds</t>
-        </is>
+          <t>Steve Such</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>217</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>295</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Premiership</t>
+          <t>Championship</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Steve Such</t>
+          <t>Jez Williams</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Jez Williams</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>213</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>287</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>20</v>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Mark Jackson</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>204</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>279</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>League One</t>
+          <t>League Two</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Mark Jackson</t>
+          <t>Carl Rowe</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>279</v>
+        <v>255</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>League Two</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Carl Rowe</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>201</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>255</v>
-      </c>
-      <c r="E17" s="7" t="n">
         <v>14</v>
       </c>
     </row>
@@ -770,7 +763,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Snakes</t>
         </is>
@@ -778,174 +771,174 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Paul Chapman</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Gary Adcock</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Camels</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Tim Lewis</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Ian Ind</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Gary Adcock</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="5" t="n">
         <v>9</v>
       </c>
     </row>
@@ -970,7 +963,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Away day credits</t>
         </is>
@@ -985,37 +978,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Weeks</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>26</v>
       </c>
       <c r="D5" s="8" t="n">
@@ -1023,15 +1016,15 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Gary Adcock</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>25</v>
       </c>
       <c r="D6" s="9" t="n">
@@ -1039,15 +1032,15 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Ian Ind</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="5" t="n">
         <v>25</v>
       </c>
       <c r="D7" s="8" t="n">
@@ -1055,15 +1048,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>25</v>
       </c>
       <c r="D8" s="9" t="n">
@@ -1071,15 +1064,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="5" t="n">
         <v>24</v>
       </c>
       <c r="D9" s="8" t="n">
@@ -1087,15 +1080,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>24</v>
       </c>
       <c r="D10" s="9" t="n">
@@ -1103,15 +1096,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Tim Lewis</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="5" t="n">
         <v>24</v>
       </c>
       <c r="D11" s="8" t="n">
@@ -1119,15 +1112,15 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>23</v>
       </c>
       <c r="D12" s="9" t="n">
@@ -1135,15 +1128,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Tony Mynard</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="5" t="n">
         <v>23</v>
       </c>
       <c r="D13" s="8" t="n">
@@ -1151,15 +1144,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Andrew Mosson</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>22</v>
       </c>
       <c r="D14" s="9" t="n">
@@ -1167,15 +1160,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Mark Jackson</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="5" t="n">
         <v>22</v>
       </c>
       <c r="D15" s="8" t="n">
@@ -1183,15 +1176,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Martin Stevenson</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>22</v>
       </c>
       <c r="D16" s="9" t="n">
@@ -1199,15 +1192,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="5" t="n">
         <v>22</v>
       </c>
       <c r="D17" s="8" t="n">
@@ -1215,15 +1208,15 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="6" t="n">
         <v>21</v>
       </c>
       <c r="D18" s="9" t="n">
@@ -1231,15 +1224,15 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="5" t="n">
         <v>21</v>
       </c>
       <c r="D19" s="8" t="n">
@@ -1247,15 +1240,15 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="6" t="n">
         <v>20</v>
       </c>
       <c r="D20" s="9" t="n">
@@ -1263,15 +1256,15 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Jez Williams</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="5" t="n">
         <v>20</v>
       </c>
       <c r="D21" s="8" t="n">
@@ -1279,15 +1272,15 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n">
+      <c r="C22" s="6" t="n">
         <v>19</v>
       </c>
       <c r="D22" s="9" t="n">
@@ -1295,15 +1288,15 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="5" t="n">
         <v>19</v>
       </c>
       <c r="D23" s="8" t="n">
@@ -1311,15 +1304,15 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="6" t="n">
         <v>18</v>
       </c>
       <c r="D24" s="9" t="n">
@@ -1327,15 +1320,15 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Ade Cooper</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C25" s="5" t="n">
         <v>17</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -1343,15 +1336,15 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Dave Harrison</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="6" t="n">
         <v>17</v>
       </c>
       <c r="D26" s="9" t="n">
@@ -1359,15 +1352,15 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Kevin Horton</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C27" s="5" t="n">
         <v>16</v>
       </c>
       <c r="D27" s="8" t="n">
@@ -1375,15 +1368,15 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n">
+      <c r="A28" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Mick Sandoz</t>
         </is>
       </c>
-      <c r="C28" s="7" t="n">
+      <c r="C28" s="6" t="n">
         <v>15</v>
       </c>
       <c r="D28" s="9" t="n">
@@ -1391,15 +1384,15 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n">
+      <c r="A29" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Paul Chapman</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="5" t="n">
         <v>15</v>
       </c>
       <c r="D29" s="8" t="n">
@@ -1407,15 +1400,15 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Richard Bird</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="6" t="n">
         <v>15</v>
       </c>
       <c r="D30" s="9" t="n">
@@ -1423,15 +1416,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Steve Robinson</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C31" s="5" t="n">
         <v>15</v>
       </c>
       <c r="D31" s="8" t="n">
@@ -1439,15 +1432,15 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="n">
+      <c r="A32" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Stuart Murdock</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="6" t="n">
         <v>15</v>
       </c>
       <c r="D32" s="9" t="n">
@@ -1455,15 +1448,15 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n">
+      <c r="A33" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="C33" s="5" t="n">
         <v>14</v>
       </c>
       <c r="D33" s="8" t="n">
@@ -1471,15 +1464,15 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="n">
+      <c r="A34" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n">
+      <c r="C34" s="6" t="n">
         <v>14</v>
       </c>
       <c r="D34" s="9" t="n">
@@ -1487,15 +1480,15 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n">
+      <c r="A35" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C35" s="5" t="n">
         <v>13</v>
       </c>
       <c r="D35" s="8" t="n">
@@ -1503,15 +1496,15 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="n">
+      <c r="A36" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Dan Conway</t>
         </is>
       </c>
-      <c r="C36" s="7" t="n">
+      <c r="C36" s="6" t="n">
         <v>13</v>
       </c>
       <c r="D36" s="9" t="n">
@@ -1519,15 +1512,15 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n">
+      <c r="A37" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Jon Boden</t>
         </is>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C37" s="5" t="n">
         <v>13</v>
       </c>
       <c r="D37" s="8" t="n">
@@ -1535,15 +1528,15 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n">
+      <c r="A38" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Les Lawrence</t>
         </is>
       </c>
-      <c r="C38" s="7" t="n">
+      <c r="C38" s="6" t="n">
         <v>13</v>
       </c>
       <c r="D38" s="9" t="n">
@@ -1551,15 +1544,15 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n">
+      <c r="A39" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Ross Kelly</t>
         </is>
       </c>
-      <c r="C39" s="6" t="n">
+      <c r="C39" s="5" t="n">
         <v>13</v>
       </c>
       <c r="D39" s="8" t="n">
@@ -1567,15 +1560,15 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="n">
+      <c r="A40" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Tom Green</t>
         </is>
       </c>
-      <c r="C40" s="7" t="n">
+      <c r="C40" s="6" t="n">
         <v>13</v>
       </c>
       <c r="D40" s="9" t="n">
@@ -1583,15 +1576,15 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Andy Ray</t>
         </is>
       </c>
-      <c r="C41" s="6" t="n">
+      <c r="C41" s="5" t="n">
         <v>12</v>
       </c>
       <c r="D41" s="8" t="n">
@@ -1599,15 +1592,15 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n">
+      <c r="A42" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>James Simmons</t>
         </is>
       </c>
-      <c r="C42" s="7" t="n">
+      <c r="C42" s="6" t="n">
         <v>12</v>
       </c>
       <c r="D42" s="9" t="n">
@@ -1615,15 +1608,15 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n">
+      <c r="A43" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Paul Smith</t>
         </is>
       </c>
-      <c r="C43" s="6" t="n">
+      <c r="C43" s="5" t="n">
         <v>12</v>
       </c>
       <c r="D43" s="8" t="n">
@@ -1631,15 +1624,15 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Jon Murchington</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n">
+      <c r="C44" s="6" t="n">
         <v>10</v>
       </c>
       <c r="D44" s="9" t="n">
@@ -1647,15 +1640,15 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n">
+      <c r="A45" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Mark Mosley</t>
         </is>
       </c>
-      <c r="C45" s="6" t="n">
+      <c r="C45" s="5" t="n">
         <v>10</v>
       </c>
       <c r="D45" s="8" t="n">
@@ -1663,15 +1656,15 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="n">
+      <c r="A46" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Stuart Pickersgill</t>
         </is>
       </c>
-      <c r="C46" s="7" t="n">
+      <c r="C46" s="6" t="n">
         <v>10</v>
       </c>
       <c r="D46" s="9" t="n">
@@ -1679,15 +1672,15 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Ashley Wells</t>
         </is>
       </c>
-      <c r="C47" s="6" t="n">
+      <c r="C47" s="5" t="n">
         <v>8</v>
       </c>
       <c r="D47" s="8" t="n">
@@ -1695,15 +1688,15 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n">
+      <c r="A48" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Paul Blades</t>
         </is>
       </c>
-      <c r="C48" s="7" t="n">
+      <c r="C48" s="6" t="n">
         <v>8</v>
       </c>
       <c r="D48" s="9" t="n">
@@ -1711,15 +1704,15 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Steve Rochester</t>
         </is>
       </c>
-      <c r="C49" s="6" t="n">
+      <c r="C49" s="5" t="n">
         <v>8</v>
       </c>
       <c r="D49" s="8" t="n">
@@ -1727,15 +1720,15 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="n">
+      <c r="A50" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>Marc Allsopp</t>
         </is>
       </c>
-      <c r="C50" s="7" t="n">
+      <c r="C50" s="6" t="n">
         <v>7</v>
       </c>
       <c r="D50" s="9" t="n">
@@ -1743,15 +1736,15 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n">
+      <c r="A51" s="5" t="n">
         <v>47</v>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Andy Spencer</t>
         </is>
       </c>
-      <c r="C51" s="6" t="n">
+      <c r="C51" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D51" s="8" t="n">
@@ -1759,15 +1752,15 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="n">
+      <c r="A52" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Richard Craven Jones</t>
         </is>
       </c>
-      <c r="C52" s="7" t="n">
+      <c r="C52" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D52" s="9" t="n">
@@ -1775,15 +1768,15 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n">
+      <c r="A53" s="5" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Richard Cook</t>
         </is>
       </c>
-      <c r="C53" s="6" t="n">
+      <c r="C53" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D53" s="8" t="n">
@@ -1791,15 +1784,15 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="n">
+      <c r="A54" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>Brian Elliot</t>
         </is>
       </c>
-      <c r="C54" s="7" t="n">
+      <c r="C54" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D54" s="9" t="n">
@@ -1807,15 +1800,15 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n">
+      <c r="A55" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Mark Jeffries</t>
         </is>
       </c>
-      <c r="C55" s="6" t="n">
+      <c r="C55" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D55" s="8" t="n">
@@ -1823,15 +1816,15 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="n">
+      <c r="A56" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Mick Hennessy</t>
         </is>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C56" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D56" s="9" t="n">
@@ -1871,7 +1864,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Champions League field</t>
         </is>
@@ -1879,98 +1872,98 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
@@ -1978,7 +1971,7 @@
     </row>
     <row r="17"/>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>RS Cup</t>
         </is>
@@ -1993,36 +1986,36 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Semi-final</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Winner</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Mark Ready vs Steve Such</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Simon Carter vs Ade Cooper</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>
@@ -2048,7 +2041,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Money summary</t>
         </is>
@@ -2063,29 +2056,29 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Entry fees collected</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>£5.00 × 784 games</t>
         </is>
@@ -2095,12 +2088,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Snake &amp; camel fines</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>£1.00 × 404</t>
         </is>
@@ -2121,12 +2114,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Weekly winner payouts</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Champions League — outright weekly winners</t>
         </is>
@@ -2136,12 +2129,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Final week split</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Shared among top scores — no Champions place</t>
         </is>
@@ -2151,12 +2144,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Club bank</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>£3.50 per game (£2744.00) + fines (£404.00)</t>
         </is>
@@ -2181,12 +2174,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Away day credits</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>£1.50 per week played · 784 games</t>
         </is>
@@ -2218,7 +2211,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
@@ -2226,392 +2219,392 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Rounds</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>295</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="5" t="n">
         <v>217</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Jez Williams</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>287</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Mark Jackson</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>279</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>204</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>278</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>277</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>207</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>275</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>273</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>207</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>273</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="n">
         <v>201</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>272</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>271</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="n">
         <v>202</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>270</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="5" t="n">
         <v>199</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>263</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Andrew Mosson</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="5" t="n">
         <v>263</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="5" t="n">
         <v>199</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Ian Ind</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="6" t="n">
         <v>262</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <v>193</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="5" t="n">
         <v>261</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="5" t="n">
         <v>195</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
@@ -2639,7 +2632,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
@@ -2647,314 +2640,314 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Rounds</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>217</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="5" t="n">
         <v>295</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="5" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>207</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="6" t="n">
         <v>277</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="6" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>207</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>273</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Simon Carter</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <v>275</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="6" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>203</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>278</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>199</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>270</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="6" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Tony Mynard</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>196</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>261</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Ian Ind</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>193</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="n">
         <v>262</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="6" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Dave Harrison</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="5" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Tim Lewis</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="n">
         <v>251</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="6" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Richard Bird</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>184</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="5" t="n">
         <v>235</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Jon Boden</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>209</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Andy Ray</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="5" t="n">
         <v>199</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="6" t="n">
         <v>176</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <v>218</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Tom Green</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="5" t="n">
         <v>151</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="5" t="n">
         <v>173</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="5" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2980,7 +2973,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
@@ -2988,314 +2981,314 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Rounds</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Jez Williams</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>213</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="5" t="n">
         <v>287</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="5" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>202</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="6" t="n">
         <v>271</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="6" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>201</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>273</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <v>272</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="6" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Martin Stevenson</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>194</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>260</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Kevin Horton</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>191</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>257</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="6" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Mick Sandoz</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>191</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>249</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Steve Robinson</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>188</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>187</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>220</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="5" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Gary Adcock</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>187</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="n">
         <v>252</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="6" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Paul Smith</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>173</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="5" t="n">
         <v>197</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Jon Murchington</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>152</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>152</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Paul Blades</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="5" t="n">
         <v>133</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="5" t="n">
         <v>133</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Marc Allsopp</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="6" t="n">
         <v>104</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <v>104</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="6" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Lee Eastoe</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3321,7 +3314,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
@@ -3329,314 +3322,314 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Rounds</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Mark Jackson</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>204</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="5" t="n">
         <v>279</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="5" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="6" t="n">
         <v>263</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="6" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>195</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>261</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>194</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <v>261</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="6" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Ade Cooper</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>187</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>245</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Stuart Murdock</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>238</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="6" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Paul Chapman</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>167</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>217</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Les Lawrence</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>162</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="n">
         <v>188</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Stuart Pickersgill</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>158</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>158</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="5" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Steve Rochester</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>124</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="n">
         <v>124</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Richard Craven Jones</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Mark Jeffries</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Ross Jeffries</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Stephen Wallace</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Stu Clark</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3662,7 +3655,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
@@ -3670,428 +3663,428 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Best 14</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Rounds</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>201</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="5" t="n">
         <v>255</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="5" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Andrew Mosson</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>199</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="6" t="n">
         <v>263</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="6" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Ross Kelly</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>194</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>238</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Dan Conway</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>181</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="6" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>James Simmons</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>170</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>194</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Mark Mosley</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>166</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Ashley Wells</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>146</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>146</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Andy Spencer</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Richard Cook</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="5" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Brian Elliot</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Mick Hennessy</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Craig Jones</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Craig Milligan</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>James Willis</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n">
+      <c r="C17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Jon Price</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Matt Spencer</t>
         </is>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="E19" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Neale Aston</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E20" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Paul Garratt</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="E21" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Scott Worrall</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="6" t="n">
+      <c r="E22" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Steve Tarmey</t>
         </is>
       </c>
-      <c r="C23" s="7" t="n">
+      <c r="C23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="E23" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Warren Crook</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="6" t="n">
+      <c r="E24" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4116,7 +4109,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>2027 promotion &amp; relegation</t>
         </is>
@@ -4124,421 +4117,421 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Promoted</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Jez Williams</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="5" t="n">
         <v>213</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Richard Shaw</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="6" t="n">
         <v>202</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="5" t="n">
         <v>201</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Mark Jackson</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="6" t="n">
         <v>204</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="5" t="n">
         <v>198</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="6" t="n">
         <v>195</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="5" t="n">
         <v>201</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Andrew Mosson</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="6" t="n">
         <v>199</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Ross Kelly</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="5" t="n">
         <v>194</v>
       </c>
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Relegated</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Best 10</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Andy Ray</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="5" t="n">
         <v>176</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="6" t="n">
         <v>176</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Tom Green</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="5" t="n">
         <v>151</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Paul Blades</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="6" t="n">
         <v>133</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Marc Allsopp</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="5" t="n">
         <v>104</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Lee Eastoe</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Championship</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Ross Jeffries</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Stephen Wallace</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Stu Clark</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>League One</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>League Two</t>
         </is>
       </c>
-      <c r="D25" s="6" t="n">
+      <c r="D25" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4556,14 +4549,14 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Weekly winners</t>
         </is>
@@ -4572,43 +4565,43 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All outright Champions · 13 winners · £1095.00</t>
+          <t>All outright Champions · 13 · £1095.00</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Paid</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Carl Rowe</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="8" t="n">
@@ -4616,15 +4609,15 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Steve Such</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="9" t="n">
@@ -4632,15 +4625,15 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>James Harrison</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="8" t="n">
@@ -4648,15 +4641,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Adam Simcox</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="9" t="n">
@@ -4664,15 +4657,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Nick Stableford</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="8" t="n">
@@ -4680,15 +4673,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Peter Jeffries</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="9" t="n">
@@ -4696,15 +4689,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Mark Ready</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="8" t="n">
@@ -4712,15 +4705,15 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Chris Boards</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="9" t="n">
@@ -4728,15 +4721,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Adam Teale</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="8" t="n">
@@ -4744,15 +4737,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Mark Howell</t>
         </is>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="9" t="n">
@@ -4760,15 +4753,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Tim Allsopp</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="8" t="n">
@@ -4776,15 +4769,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>John Goodman</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="9" t="n">
@@ -4792,15 +4785,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>James Tough</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="8" t="n">

</xml_diff>